<commit_message>
Replace all files with updated versions
</commit_message>
<xml_diff>
--- a/results/validation/predictions_ all.xlsx
+++ b/results/validation/predictions_ all.xlsx
@@ -5,27 +5,36 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Николай\Documents\Работа ИФМ\Машинное обучение\ML plan\Featurization FeSiAl\статья\Результаты расчетов\Prediction_results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Niccuby\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AC408F9-E125-4AE6-8DD9-CB6A5F72AE5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8360B1C-E9FC-4760-B020-07E0861D056D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1815" yWindow="1815" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="23">
   <si>
     <t>Model</t>
   </si>
@@ -66,9 +75,6 @@
     <t>WenAlloys Resistivity</t>
   </si>
   <si>
-    <t>MAE</t>
-  </si>
-  <si>
     <t>Oliynyk Coercivity</t>
   </si>
   <si>
@@ -92,15 +98,21 @@
   <si>
     <t>Composition Resistivity</t>
   </si>
+  <si>
+    <t>AE</t>
+  </si>
+  <si>
+    <t>APE</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -127,8 +139,17 @@
       <family val="2"/>
       <charset val="204"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -162,6 +183,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE4C9FF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -310,7 +337,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -330,16 +357,16 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -355,12 +382,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFE4C9FF"/>
+      <color rgb="FFCC99FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -636,46 +671,46 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B3:AE45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" customWidth="1"/>
-    <col min="8" max="8" width="23.28515625" customWidth="1"/>
+    <col min="7" max="7" width="11.5546875" customWidth="1"/>
+    <col min="8" max="8" width="23.33203125" customWidth="1"/>
     <col min="13" max="13" width="14" customWidth="1"/>
     <col min="14" max="14" width="13" customWidth="1"/>
-    <col min="15" max="15" width="9.28515625" customWidth="1"/>
-    <col min="17" max="17" width="12.7109375" customWidth="1"/>
-    <col min="18" max="18" width="20.85546875" customWidth="1"/>
-    <col min="22" max="22" width="13.7109375" customWidth="1"/>
-    <col min="23" max="23" width="13.42578125" customWidth="1"/>
+    <col min="15" max="15" width="9.33203125" customWidth="1"/>
+    <col min="17" max="17" width="12.6640625" customWidth="1"/>
+    <col min="18" max="18" width="20.88671875" customWidth="1"/>
+    <col min="22" max="22" width="13.6640625" customWidth="1"/>
+    <col min="23" max="23" width="13.44140625" customWidth="1"/>
     <col min="24" max="24" width="13" customWidth="1"/>
     <col min="27" max="27" width="12" customWidth="1"/>
-    <col min="28" max="28" width="21.140625" customWidth="1"/>
+    <col min="28" max="28" width="21.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:31" ht="18.75" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:31" ht="17.399999999999999" x14ac:dyDescent="0.45">
       <c r="D3" s="29" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E3" s="30"/>
       <c r="F3" s="30"/>
       <c r="G3" s="31"/>
       <c r="N3" s="29" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O3" s="30"/>
       <c r="P3" s="30"/>
       <c r="Q3" s="31"/>
       <c r="X3" s="29" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="Y3" s="30"/>
       <c r="Z3" s="30"/>
       <c r="AA3" s="31"/>
     </row>
-    <row r="4" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
@@ -689,13 +724,13 @@
         <v>3</v>
       </c>
       <c r="F4" s="28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G4" s="28" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="H4" s="28" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="L4" s="1" t="s">
         <v>0</v>
@@ -710,13 +745,13 @@
         <v>7</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q4" s="28" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="R4" s="28" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="V4" s="28" t="s">
         <v>0</v>
@@ -731,17 +766,17 @@
         <v>9</v>
       </c>
       <c r="Z4" s="28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="AA4" s="28" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="AB4" s="28" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="AE4" s="27"/>
     </row>
-    <row r="5" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
@@ -749,19 +784,19 @@
         <v>1</v>
       </c>
       <c r="D5" s="17">
-        <v>4.1246</v>
+        <v>4.1455500000000018</v>
       </c>
       <c r="E5" s="17">
         <v>5.6</v>
       </c>
       <c r="F5" s="17">
-        <v>-1.4754</v>
+        <v>-1.454449999999998</v>
       </c>
       <c r="G5" s="17">
-        <v>1.4754</v>
+        <v>1.454449999999998</v>
       </c>
       <c r="H5" s="18">
-        <v>26.346428571428572</v>
+        <v>25.972321428571391</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>4</v>
@@ -770,19 +805,19 @@
         <v>1</v>
       </c>
       <c r="N5" s="4">
-        <v>1.1047002301123721</v>
+        <v>1.1087830132140919</v>
       </c>
       <c r="O5" s="4">
         <v>0.93700000000000006</v>
       </c>
       <c r="P5" s="4">
-        <v>0.1677002301123722</v>
+        <v>0.17178301321409181</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.1677002301123722</v>
+        <v>0.17178301321409181</v>
       </c>
       <c r="R5" s="18">
-        <v>17.897569915941538</v>
+        <v>18.333299169059959</v>
       </c>
       <c r="V5" s="2" t="s">
         <v>4</v>
@@ -791,22 +826,22 @@
         <v>1</v>
       </c>
       <c r="X5" s="17">
-        <v>81.516940789473651</v>
+        <v>80.705098684210427</v>
       </c>
       <c r="Y5" s="17">
         <v>86.8</v>
       </c>
       <c r="Z5" s="17">
-        <v>-5.2830592105263463</v>
+        <v>-6.0949013157895706</v>
       </c>
       <c r="AA5" s="17">
-        <v>5.2830592105263463</v>
+        <v>6.0949013157895706</v>
       </c>
       <c r="AB5" s="18">
-        <v>6.0864737448460211</v>
-      </c>
-    </row>
-    <row r="6" spans="2:31" x14ac:dyDescent="0.25">
+        <v>7.0217757094349897</v>
+      </c>
+    </row>
+    <row r="6" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>4</v>
       </c>
@@ -814,19 +849,19 @@
         <v>2</v>
       </c>
       <c r="D6" s="19">
-        <v>3.6272249999999979</v>
+        <v>3.4337500000000012</v>
       </c>
       <c r="E6" s="19">
         <v>5.47</v>
       </c>
       <c r="F6" s="19">
-        <v>-1.8427750000000009</v>
+        <v>-2.036249999999999</v>
       </c>
       <c r="G6" s="19">
-        <v>1.8427750000000009</v>
+        <v>2.036249999999999</v>
       </c>
       <c r="H6" s="20">
-        <v>33.688756855575903</v>
+        <v>37.225776965265062</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>4</v>
@@ -835,19 +870,19 @@
         <v>2</v>
       </c>
       <c r="N6" s="7">
-        <v>0.89690381845818157</v>
+        <v>0.89312970119688895</v>
       </c>
       <c r="O6" s="7">
         <v>0.88400000000000001</v>
       </c>
       <c r="P6" s="7">
-        <v>1.290381845818156E-2</v>
+        <v>9.1297011968889397E-3</v>
       </c>
       <c r="Q6" s="7">
-        <v>1.290381845818156E-2</v>
+        <v>9.1297011968889397E-3</v>
       </c>
       <c r="R6" s="20">
-        <v>1.4597079703825291</v>
+        <v>1.0327716286073461</v>
       </c>
       <c r="V6" s="5" t="s">
         <v>4</v>
@@ -856,22 +891,22 @@
         <v>2</v>
       </c>
       <c r="X6" s="19">
-        <v>103.8705592105263</v>
+        <v>104.68388157894729</v>
       </c>
       <c r="Y6" s="19">
         <v>106.9</v>
       </c>
       <c r="Z6" s="19">
-        <v>-3.029440789473739</v>
+        <v>-2.2161184210526979</v>
       </c>
       <c r="AA6" s="19">
-        <v>3.029440789473739</v>
+        <v>2.2161184210526979</v>
       </c>
       <c r="AB6" s="20">
-        <v>2.8339015804244521</v>
-      </c>
-    </row>
-    <row r="7" spans="2:31" x14ac:dyDescent="0.25">
+        <v>2.0730761656246011</v>
+      </c>
+    </row>
+    <row r="7" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B7" s="8" t="s">
         <v>4</v>
       </c>
@@ -879,19 +914,19 @@
         <v>3</v>
       </c>
       <c r="D7" s="21">
-        <v>12.27387500000002</v>
+        <v>11.789849999999999</v>
       </c>
       <c r="E7" s="21">
         <v>26.16</v>
       </c>
       <c r="F7" s="21">
-        <v>-13.88612499999998</v>
+        <v>-14.370150000000001</v>
       </c>
       <c r="G7" s="21">
-        <v>13.88612499999998</v>
+        <v>14.370150000000001</v>
       </c>
       <c r="H7" s="22">
-        <v>53.081517584097803</v>
+        <v>54.931766055045863</v>
       </c>
       <c r="L7" s="8" t="s">
         <v>4</v>
@@ -900,19 +935,19 @@
         <v>3</v>
       </c>
       <c r="N7" s="10">
-        <v>0.6430184502923969</v>
+        <v>0.64722810846560797</v>
       </c>
       <c r="O7" s="10">
         <v>0.60699999999999998</v>
       </c>
       <c r="P7" s="10">
-        <v>3.601845029239692E-2</v>
+        <v>4.0228108465607981E-2</v>
       </c>
       <c r="Q7" s="10">
-        <v>3.601845029239692E-2</v>
+        <v>4.0228108465607981E-2</v>
       </c>
       <c r="R7" s="22">
-        <v>5.9338468356502343</v>
+        <v>6.6273654803308046</v>
       </c>
       <c r="V7" s="8" t="s">
         <v>4</v>
@@ -921,22 +956,22 @@
         <v>3</v>
       </c>
       <c r="X7" s="21">
-        <v>134.07467105263129</v>
+        <v>132.8223684210522</v>
       </c>
       <c r="Y7" s="21">
         <v>146.1</v>
       </c>
       <c r="Z7" s="21">
-        <v>-12.02532894736871</v>
+        <v>-13.27763157894776</v>
       </c>
       <c r="AA7" s="21">
-        <v>12.02532894736871</v>
+        <v>13.27763157894776</v>
       </c>
       <c r="AB7" s="22">
-        <v>8.2308890810189652</v>
-      </c>
-    </row>
-    <row r="8" spans="2:31" x14ac:dyDescent="0.25">
+        <v>9.0880435174180434</v>
+      </c>
+    </row>
+    <row r="8" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B8" s="11" t="s">
         <v>4</v>
       </c>
@@ -944,19 +979,22 @@
         <v>4</v>
       </c>
       <c r="D8" s="23">
-        <v>25.445199999999989</v>
+        <v>24.581074999999998</v>
       </c>
       <c r="E8" s="23">
         <v>47.29</v>
       </c>
       <c r="F8" s="23">
-        <v>-21.84480000000001</v>
+        <v>-22.708925000000001</v>
       </c>
       <c r="G8" s="23">
-        <v>21.84480000000001</v>
+        <v>22.708925000000001</v>
       </c>
       <c r="H8" s="24">
-        <v>46.193275533939541</v>
+        <v>48.020564601395641</v>
+      </c>
+      <c r="I8" s="32" t="s">
+        <v>17</v>
       </c>
       <c r="L8" s="11" t="s">
         <v>4</v>
@@ -965,19 +1003,22 @@
         <v>4</v>
       </c>
       <c r="N8" s="13">
-        <v>0.81045487004548411</v>
+        <v>0.74929366963283794</v>
       </c>
       <c r="O8" s="13">
         <v>0.79400000000000004</v>
       </c>
       <c r="P8" s="13">
-        <v>1.6454870045484071E-2</v>
+        <v>-4.4706330367162088E-2</v>
       </c>
       <c r="Q8" s="13">
-        <v>1.6454870045484071E-2</v>
+        <v>4.4706330367162088E-2</v>
       </c>
       <c r="R8" s="24">
-        <v>2.0724017689526542</v>
+        <v>5.6305201973755787</v>
+      </c>
+      <c r="S8" s="32" t="s">
+        <v>17</v>
       </c>
       <c r="V8" s="11" t="s">
         <v>4</v>
@@ -986,22 +1027,25 @@
         <v>4</v>
       </c>
       <c r="X8" s="23">
-        <v>100.3179276315788</v>
+        <v>101.1710526315788</v>
       </c>
       <c r="Y8" s="23">
         <v>122.8</v>
       </c>
       <c r="Z8" s="23">
-        <v>-22.482072368421171</v>
+        <v>-21.62894736842118</v>
       </c>
       <c r="AA8" s="23">
-        <v>22.482072368421171</v>
+        <v>21.62894736842118</v>
       </c>
       <c r="AB8" s="24">
-        <v>18.30787652151561</v>
-      </c>
-    </row>
-    <row r="9" spans="2:31" x14ac:dyDescent="0.25">
+        <v>17.613149322818551</v>
+      </c>
+      <c r="AC8" s="32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B9" s="14" t="s">
         <v>4</v>
       </c>
@@ -1009,19 +1053,23 @@
         <v>5</v>
       </c>
       <c r="D9" s="25">
-        <v>14.34440000000003</v>
+        <v>14.25117500000003</v>
       </c>
       <c r="E9" s="25">
         <v>26.24</v>
       </c>
       <c r="F9" s="25">
-        <v>-11.89559999999997</v>
+        <v>-11.98882499999997</v>
       </c>
       <c r="G9" s="25">
-        <v>11.89559999999997</v>
+        <v>11.98882499999997</v>
       </c>
       <c r="H9" s="26">
-        <v>45.333841463414522</v>
+        <v>45.689119664634028</v>
+      </c>
+      <c r="I9" s="33">
+        <f>AVERAGE(H5:H9)</f>
+        <v>42.367909742982398</v>
       </c>
       <c r="L9" s="14" t="s">
         <v>4</v>
@@ -1030,19 +1078,23 @@
         <v>5</v>
       </c>
       <c r="N9" s="16">
-        <v>1.672119026241248</v>
+        <v>1.6694450934970371</v>
       </c>
       <c r="O9" s="16">
         <v>1.5740000000000001</v>
       </c>
       <c r="P9" s="16">
-        <v>9.8119026241247687E-2</v>
+        <v>9.5445093497037004E-2</v>
       </c>
       <c r="Q9" s="16">
-        <v>9.8119026241247687E-2</v>
+        <v>9.5445093497037004E-2</v>
       </c>
       <c r="R9" s="26">
-        <v>6.2337373723791414</v>
+        <v>6.0638560036236973</v>
+      </c>
+      <c r="S9" s="33">
+        <f>AVERAGE(R5:R9)</f>
+        <v>7.5375624957994773</v>
       </c>
       <c r="V9" s="14" t="s">
         <v>4</v>
@@ -1051,22 +1103,26 @@
         <v>5</v>
       </c>
       <c r="X9" s="25">
-        <v>93.8666118421053</v>
+        <v>93.364967105263275</v>
       </c>
       <c r="Y9" s="25">
         <v>101.2</v>
       </c>
       <c r="Z9" s="25">
-        <v>-7.3333881578947029</v>
+        <v>-7.8350328947367274</v>
       </c>
       <c r="AA9" s="25">
-        <v>7.3333881578947029</v>
+        <v>7.8350328947367274</v>
       </c>
       <c r="AB9" s="26">
-        <v>7.2464309860619593</v>
-      </c>
-    </row>
-    <row r="10" spans="2:31" x14ac:dyDescent="0.25">
+        <v>7.7421273663406396</v>
+      </c>
+      <c r="AC9" s="33">
+        <f>AVERAGE(AB5:AB9)</f>
+        <v>8.7076344163273642</v>
+      </c>
+    </row>
+    <row r="10" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B10" s="2" t="s">
         <v>5</v>
       </c>
@@ -1074,19 +1130,19 @@
         <v>1</v>
       </c>
       <c r="D10" s="17">
-        <v>4.297515869140625</v>
+        <v>5.1913914680480957</v>
       </c>
       <c r="E10" s="17">
         <v>5.6</v>
       </c>
       <c r="F10" s="17">
-        <v>-1.3024841308593751</v>
+        <v>-0.40860853195190389</v>
       </c>
       <c r="G10" s="17">
-        <v>1.3024841308593751</v>
+        <v>0.40860853195190389</v>
       </c>
       <c r="H10" s="18">
-        <v>23.25864519391741</v>
+        <v>7.2965809277125704</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>5</v>
@@ -1095,19 +1151,19 @@
         <v>1</v>
       </c>
       <c r="N10" s="4">
-        <v>1.141227126121521</v>
+        <v>1.105050206184387</v>
       </c>
       <c r="O10" s="4">
         <v>0.93700000000000006</v>
       </c>
       <c r="P10" s="4">
-        <v>0.20422712612152091</v>
+        <v>0.16805020618438721</v>
       </c>
       <c r="Q10" s="4">
-        <v>0.20422712612152091</v>
+        <v>0.16805020618438721</v>
       </c>
       <c r="R10" s="18">
-        <v>21.795851240290389</v>
+        <v>17.93492061733054</v>
       </c>
       <c r="V10" s="2" t="s">
         <v>5</v>
@@ -1116,22 +1172,22 @@
         <v>1</v>
       </c>
       <c r="X10" s="17">
-        <v>73.602088928222656</v>
+        <v>74.578804016113281</v>
       </c>
       <c r="Y10" s="17">
         <v>86.8</v>
       </c>
       <c r="Z10" s="17">
-        <v>-13.197911071777339</v>
+        <v>-12.221195983886719</v>
       </c>
       <c r="AA10" s="17">
-        <v>13.197911071777339</v>
+        <v>12.221195983886719</v>
       </c>
       <c r="AB10" s="18">
-        <v>15.204966672554541</v>
-      </c>
-    </row>
-    <row r="11" spans="2:31" x14ac:dyDescent="0.25">
+        <v>14.079718875445529</v>
+      </c>
+    </row>
+    <row r="11" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B11" s="5" t="s">
         <v>5</v>
       </c>
@@ -1139,19 +1195,19 @@
         <v>2</v>
       </c>
       <c r="D11" s="19">
-        <v>4.1074151992797852</v>
+        <v>3.6597917079925542</v>
       </c>
       <c r="E11" s="19">
         <v>5.47</v>
       </c>
       <c r="F11" s="19">
-        <v>-1.362584800720215</v>
+        <v>-1.810208292007446</v>
       </c>
       <c r="G11" s="19">
-        <v>1.362584800720215</v>
+        <v>1.810208292007446</v>
       </c>
       <c r="H11" s="20">
-        <v>24.910142609144689</v>
+        <v>33.093387422439598</v>
       </c>
       <c r="L11" s="5" t="s">
         <v>5</v>
@@ -1160,19 +1216,19 @@
         <v>2</v>
       </c>
       <c r="N11" s="7">
-        <v>0.88466018438339233</v>
+        <v>0.91320818662643433</v>
       </c>
       <c r="O11" s="7">
         <v>0.88400000000000001</v>
       </c>
       <c r="P11" s="7">
-        <v>6.6018438339232599E-4</v>
+        <v>2.9208186626434322E-2</v>
       </c>
       <c r="Q11" s="7">
-        <v>6.6018438339232599E-4</v>
+        <v>2.9208186626434322E-2</v>
       </c>
       <c r="R11" s="20">
-        <v>7.4681491333973532E-2</v>
+        <v>3.3040935097776378</v>
       </c>
       <c r="V11" s="5" t="s">
         <v>5</v>
@@ -1181,22 +1237,22 @@
         <v>2</v>
       </c>
       <c r="X11" s="19">
-        <v>103.3385848999023</v>
+        <v>103.7990036010742</v>
       </c>
       <c r="Y11" s="19">
         <v>106.9</v>
       </c>
       <c r="Z11" s="19">
-        <v>-3.5614151000976619</v>
+        <v>-3.1009963989257869</v>
       </c>
       <c r="AA11" s="19">
-        <v>3.5614151000976619</v>
+        <v>3.1009963989257869</v>
       </c>
       <c r="AB11" s="20">
-        <v>3.3315389149650718</v>
-      </c>
-    </row>
-    <row r="12" spans="2:31" x14ac:dyDescent="0.25">
+        <v>2.9008385396873591</v>
+      </c>
+    </row>
+    <row r="12" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B12" s="8" t="s">
         <v>5</v>
       </c>
@@ -1204,19 +1260,19 @@
         <v>3</v>
       </c>
       <c r="D12" s="21">
-        <v>14.406088829040529</v>
+        <v>14.289290428161619</v>
       </c>
       <c r="E12" s="21">
         <v>26.16</v>
       </c>
       <c r="F12" s="21">
-        <v>-11.753911170959469</v>
+        <v>-11.870709571838381</v>
       </c>
       <c r="G12" s="21">
-        <v>11.753911170959469</v>
+        <v>11.870709571838381</v>
       </c>
       <c r="H12" s="22">
-        <v>44.930853099997982</v>
+        <v>45.377330167577902</v>
       </c>
       <c r="L12" s="8" t="s">
         <v>5</v>
@@ -1225,19 +1281,19 @@
         <v>3</v>
       </c>
       <c r="N12" s="10">
-        <v>0.56212395429611206</v>
+        <v>0.52593940496444702</v>
       </c>
       <c r="O12" s="10">
         <v>0.60699999999999998</v>
       </c>
       <c r="P12" s="10">
-        <v>-4.4876045703887923E-2</v>
+        <v>-8.1060595035552963E-2</v>
       </c>
       <c r="Q12" s="10">
-        <v>4.4876045703887923E-2</v>
+        <v>8.1060595035552963E-2</v>
       </c>
       <c r="R12" s="22">
-        <v>7.3930882543472691</v>
+        <v>13.354299017389289</v>
       </c>
       <c r="V12" s="8" t="s">
         <v>5</v>
@@ -1246,22 +1302,22 @@
         <v>3</v>
       </c>
       <c r="X12" s="21">
-        <v>140.19056701660159</v>
+        <v>135.2191162109375</v>
       </c>
       <c r="Y12" s="21">
         <v>146.1</v>
       </c>
       <c r="Z12" s="21">
-        <v>-5.9094329833984318</v>
+        <v>-10.880883789062491</v>
       </c>
       <c r="AA12" s="21">
-        <v>5.9094329833984318</v>
+        <v>10.880883789062491</v>
       </c>
       <c r="AB12" s="22">
-        <v>4.0447864362754498</v>
-      </c>
-    </row>
-    <row r="13" spans="2:31" x14ac:dyDescent="0.25">
+        <v>7.4475590616444176</v>
+      </c>
+    </row>
+    <row r="13" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B13" s="11" t="s">
         <v>5</v>
       </c>
@@ -1269,19 +1325,22 @@
         <v>4</v>
       </c>
       <c r="D13" s="23">
-        <v>37.599876403808587</v>
+        <v>29.12613677978516</v>
       </c>
       <c r="E13" s="23">
         <v>47.29</v>
       </c>
       <c r="F13" s="23">
-        <v>-9.6901235961914054</v>
+        <v>-18.163863220214839</v>
       </c>
       <c r="G13" s="23">
-        <v>9.6901235961914054</v>
+        <v>18.163863220214839</v>
       </c>
       <c r="H13" s="24">
-        <v>20.490851334724901</v>
+        <v>38.409522563364021</v>
+      </c>
+      <c r="I13" s="32" t="s">
+        <v>17</v>
       </c>
       <c r="L13" s="11" t="s">
         <v>5</v>
@@ -1290,19 +1349,22 @@
         <v>4</v>
       </c>
       <c r="N13" s="13">
-        <v>0.67794746160507202</v>
+        <v>0.67040115594863892</v>
       </c>
       <c r="O13" s="13">
         <v>0.79400000000000004</v>
       </c>
       <c r="P13" s="13">
-        <v>-0.116052538394928</v>
+        <v>-0.1235988440513611</v>
       </c>
       <c r="Q13" s="13">
-        <v>0.116052538394928</v>
+        <v>0.1235988440513611</v>
       </c>
       <c r="R13" s="24">
-        <v>14.61618871472645</v>
+        <v>15.566605044252031</v>
+      </c>
+      <c r="S13" s="32" t="s">
+        <v>17</v>
       </c>
       <c r="V13" s="11" t="s">
         <v>5</v>
@@ -1311,22 +1373,25 @@
         <v>4</v>
       </c>
       <c r="X13" s="23">
-        <v>109.3234786987305</v>
+        <v>107.89865875244141</v>
       </c>
       <c r="Y13" s="23">
         <v>122.8</v>
       </c>
       <c r="Z13" s="23">
-        <v>-13.47652130126953</v>
+        <v>-14.901341247558589</v>
       </c>
       <c r="AA13" s="23">
-        <v>13.47652130126953</v>
+        <v>14.901341247558589</v>
       </c>
       <c r="AB13" s="24">
-        <v>10.97436588051265</v>
-      </c>
-    </row>
-    <row r="14" spans="2:31" x14ac:dyDescent="0.25">
+        <v>12.134642709738269</v>
+      </c>
+      <c r="AC13" s="32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B14" s="14" t="s">
         <v>5</v>
       </c>
@@ -1334,19 +1399,23 @@
         <v>5</v>
       </c>
       <c r="D14" s="25">
-        <v>12.47068881988525</v>
+        <v>12.841836929321291</v>
       </c>
       <c r="E14" s="25">
         <v>26.24</v>
       </c>
       <c r="F14" s="25">
-        <v>-13.769311180114739</v>
+        <v>-13.398163070678709</v>
       </c>
       <c r="G14" s="25">
-        <v>13.769311180114739</v>
+        <v>13.398163070678709</v>
       </c>
       <c r="H14" s="26">
-        <v>52.474509070559243</v>
+        <v>51.060072677891426</v>
+      </c>
+      <c r="I14" s="33">
+        <f>AVERAGE(H10:H14)</f>
+        <v>35.047378751797098</v>
       </c>
       <c r="L14" s="14" t="s">
         <v>5</v>
@@ -1355,19 +1424,23 @@
         <v>5</v>
       </c>
       <c r="N14" s="16">
-        <v>1.6512594223022461</v>
+        <v>1.622699379920959</v>
       </c>
       <c r="O14" s="16">
         <v>1.5740000000000001</v>
       </c>
       <c r="P14" s="16">
-        <v>7.7259422302246028E-2</v>
+        <v>4.8699379920959407E-2</v>
       </c>
       <c r="Q14" s="16">
-        <v>7.7259422302246028E-2</v>
+        <v>4.8699379920959407E-2</v>
       </c>
       <c r="R14" s="26">
-        <v>4.9084766392786543</v>
+        <v>3.0939885591460872</v>
+      </c>
+      <c r="S14" s="33">
+        <f>AVERAGE(R10:R14)</f>
+        <v>10.650781349579116</v>
       </c>
       <c r="V14" s="14" t="s">
         <v>5</v>
@@ -1376,22 +1449,26 @@
         <v>5</v>
       </c>
       <c r="X14" s="25">
-        <v>94.125167846679688</v>
+        <v>94.948944091796875</v>
       </c>
       <c r="Y14" s="25">
         <v>101.2</v>
       </c>
       <c r="Z14" s="25">
-        <v>-7.0748321533203153</v>
+        <v>-6.2510559082031278</v>
       </c>
       <c r="AA14" s="25">
-        <v>7.0748321533203153</v>
+        <v>6.2510559082031278</v>
       </c>
       <c r="AB14" s="26">
-        <v>6.990940862964738</v>
-      </c>
-    </row>
-    <row r="19" spans="2:28" ht="18.75" x14ac:dyDescent="0.4">
+        <v>6.1769327156157381</v>
+      </c>
+      <c r="AC14" s="33">
+        <f>AVERAGE(AB10:AB14)</f>
+        <v>8.5479383804262632</v>
+      </c>
+    </row>
+    <row r="19" spans="2:29" ht="17.399999999999999" x14ac:dyDescent="0.45">
       <c r="D19" s="29" t="s">
         <v>10</v>
       </c>
@@ -1411,7 +1488,7 @@
       <c r="Z19" s="30"/>
       <c r="AA19" s="31"/>
     </row>
-    <row r="20" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
         <v>0</v>
       </c>
@@ -1425,13 +1502,13 @@
         <v>3</v>
       </c>
       <c r="F20" s="28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G20" s="28" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="H20" s="28" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="L20" s="1" t="s">
         <v>0</v>
@@ -1446,13 +1523,13 @@
         <v>7</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q20" s="28" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="R20" s="28" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="V20" s="1" t="s">
         <v>0</v>
@@ -1467,16 +1544,16 @@
         <v>9</v>
       </c>
       <c r="Z20" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="AA20" s="28" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="AB20" s="28" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" spans="2:28" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B21" s="2" t="s">
         <v>4</v>
       </c>
@@ -1484,19 +1561,19 @@
         <v>1</v>
       </c>
       <c r="D21" s="17">
-        <v>3.3821499999999949</v>
+        <v>3.6131249999999988</v>
       </c>
       <c r="E21" s="17">
         <v>5.6</v>
       </c>
       <c r="F21" s="17">
-        <v>-2.2178500000000039</v>
+        <v>-1.9868749999999999</v>
       </c>
       <c r="G21" s="17">
-        <v>2.2178500000000039</v>
+        <v>1.9868749999999999</v>
       </c>
       <c r="H21" s="18">
-        <v>39.604464285714357</v>
+        <v>35.479910714285722</v>
       </c>
       <c r="L21" s="2" t="s">
         <v>4</v>
@@ -1505,19 +1582,19 @@
         <v>1</v>
       </c>
       <c r="N21" s="4">
-        <v>1.073003130511464</v>
+        <v>1.083628327454438</v>
       </c>
       <c r="O21" s="4">
         <v>0.93700000000000006</v>
       </c>
       <c r="P21" s="4">
-        <v>0.1360031305114644</v>
+        <v>0.14662832745443799</v>
       </c>
       <c r="Q21" s="4">
-        <v>0.1360031305114644</v>
+        <v>0.14662832745443799</v>
       </c>
       <c r="R21" s="18">
-        <v>14.514741783507411</v>
+        <v>15.64870090228794</v>
       </c>
       <c r="V21" s="2" t="s">
         <v>4</v>
@@ -1526,22 +1603,22 @@
         <v>1</v>
       </c>
       <c r="X21" s="17">
-        <v>80.237664473684177</v>
+        <v>80.887171052631587</v>
       </c>
       <c r="Y21" s="3">
         <v>86.8</v>
       </c>
       <c r="Z21" s="17">
-        <v>-6.5623355263158203</v>
+        <v>-5.9128289473684106</v>
       </c>
       <c r="AA21" s="17">
-        <v>6.5623355263158203</v>
+        <v>5.9128289473684106</v>
       </c>
       <c r="AB21" s="18">
-        <v>7.5602943851564746</v>
-      </c>
-    </row>
-    <row r="22" spans="2:28" x14ac:dyDescent="0.25">
+        <v>6.8120149163230526</v>
+      </c>
+    </row>
+    <row r="22" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B22" s="5" t="s">
         <v>4</v>
       </c>
@@ -1549,19 +1626,19 @@
         <v>2</v>
       </c>
       <c r="D22" s="19">
-        <v>3.9469749999999961</v>
+        <v>3.7007000000000021</v>
       </c>
       <c r="E22" s="19">
         <v>5.47</v>
       </c>
       <c r="F22" s="19">
-        <v>-1.5230250000000041</v>
+        <v>-1.7692999999999981</v>
       </c>
       <c r="G22" s="19">
-        <v>1.5230250000000041</v>
+        <v>1.7692999999999981</v>
       </c>
       <c r="H22" s="20">
-        <v>27.843235831809942</v>
+        <v>32.345521023765947</v>
       </c>
       <c r="L22" s="5" t="s">
         <v>4</v>
@@ -1570,19 +1647,19 @@
         <v>2</v>
       </c>
       <c r="N22" s="7">
-        <v>0.87974845679012392</v>
+        <v>0.89225438271604585</v>
       </c>
       <c r="O22" s="7">
         <v>0.88400000000000001</v>
       </c>
       <c r="P22" s="7">
-        <v>-4.2515432098760852E-3</v>
+        <v>8.2543827160458383E-3</v>
       </c>
       <c r="Q22" s="7">
-        <v>4.2515432098760852E-3</v>
+        <v>8.2543827160458383E-3</v>
       </c>
       <c r="R22" s="20">
-        <v>0.48094380202218162</v>
+        <v>0.93375370091016274</v>
       </c>
       <c r="V22" s="5" t="s">
         <v>4</v>
@@ -1591,22 +1668,22 @@
         <v>2</v>
       </c>
       <c r="X22" s="19">
-        <v>105.74523026315779</v>
+        <v>105.1333881578946</v>
       </c>
       <c r="Y22" s="6">
         <v>106.9</v>
       </c>
       <c r="Z22" s="19">
-        <v>-1.1547697368421981</v>
+        <v>-1.766611842105362</v>
       </c>
       <c r="AA22" s="19">
-        <v>1.1547697368421981</v>
+        <v>1.766611842105362</v>
       </c>
       <c r="AB22" s="20">
-        <v>1.0802336172518221</v>
-      </c>
-    </row>
-    <row r="23" spans="2:28" x14ac:dyDescent="0.25">
+        <v>1.6525835754025839</v>
+      </c>
+    </row>
+    <row r="23" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B23" s="8" t="s">
         <v>4</v>
       </c>
@@ -1614,19 +1691,19 @@
         <v>3</v>
       </c>
       <c r="D23" s="21">
-        <v>16.13600000000001</v>
+        <v>13.544350000000019</v>
       </c>
       <c r="E23" s="21">
         <v>26.16</v>
       </c>
       <c r="F23" s="21">
-        <v>-10.02399999999999</v>
+        <v>-12.615649999999979</v>
       </c>
       <c r="G23" s="21">
-        <v>10.02399999999999</v>
+        <v>12.615649999999979</v>
       </c>
       <c r="H23" s="22">
-        <v>38.318042813455619</v>
+        <v>48.224961773700223</v>
       </c>
       <c r="L23" s="8" t="s">
         <v>4</v>
@@ -1635,19 +1712,19 @@
         <v>3</v>
       </c>
       <c r="N23" s="10">
-        <v>0.60008796296296163</v>
+        <v>0.65711975308641901</v>
       </c>
       <c r="O23" s="10">
         <v>0.60699999999999998</v>
       </c>
       <c r="P23" s="10">
-        <v>-6.9120370370383544E-3</v>
+        <v>5.0119753086419028E-2</v>
       </c>
       <c r="Q23" s="10">
-        <v>6.9120370370383544E-3</v>
+        <v>5.0119753086419028E-2</v>
       </c>
       <c r="R23" s="22">
-        <v>1.138721093416533</v>
+        <v>8.2569609697560171</v>
       </c>
       <c r="V23" s="8" t="s">
         <v>4</v>
@@ -1656,22 +1733,22 @@
         <v>3</v>
       </c>
       <c r="X23" s="21">
-        <v>135.98421052631539</v>
+        <v>134.50394736842071</v>
       </c>
       <c r="Y23" s="9">
         <v>146.1</v>
       </c>
       <c r="Z23" s="21">
-        <v>-10.1157894736846</v>
+        <v>-11.59605263157931</v>
       </c>
       <c r="AA23" s="21">
-        <v>10.1157894736846</v>
+        <v>11.59605263157931</v>
       </c>
       <c r="AB23" s="22">
-        <v>6.9238805432475026</v>
-      </c>
-    </row>
-    <row r="24" spans="2:28" x14ac:dyDescent="0.25">
+        <v>7.937065456248674</v>
+      </c>
+    </row>
+    <row r="24" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B24" s="11" t="s">
         <v>4</v>
       </c>
@@ -1679,19 +1756,22 @@
         <v>4</v>
       </c>
       <c r="D24" s="23">
-        <v>18.74832500000003</v>
+        <v>17.406100000000031</v>
       </c>
       <c r="E24" s="23">
         <v>47.29</v>
       </c>
       <c r="F24" s="23">
-        <v>-28.541674999999969</v>
+        <v>-29.883899999999969</v>
       </c>
       <c r="G24" s="23">
-        <v>28.541674999999969</v>
+        <v>29.883899999999969</v>
       </c>
       <c r="H24" s="24">
-        <v>60.354567561852328</v>
+        <v>63.19285261154571</v>
+      </c>
+      <c r="I24" s="32" t="s">
+        <v>17</v>
       </c>
       <c r="L24" s="11" t="s">
         <v>4</v>
@@ -1700,19 +1780,22 @@
         <v>4</v>
       </c>
       <c r="N24" s="13">
-        <v>0.83098672839506171</v>
+        <v>0.8139932716049405</v>
       </c>
       <c r="O24" s="13">
         <v>0.79400000000000004</v>
       </c>
       <c r="P24" s="13">
-        <v>3.6986728395061667E-2</v>
+        <v>1.9993271604940469E-2</v>
       </c>
       <c r="Q24" s="13">
-        <v>3.6986728395061667E-2</v>
+        <v>1.9993271604940469E-2</v>
       </c>
       <c r="R24" s="24">
-        <v>4.6582781353981959</v>
+        <v>2.518044282738094</v>
+      </c>
+      <c r="S24" s="32" t="s">
+        <v>17</v>
       </c>
       <c r="V24" s="11" t="s">
         <v>4</v>
@@ -1721,22 +1804,25 @@
         <v>4</v>
       </c>
       <c r="X24" s="23">
-        <v>106.73388157894711</v>
+        <v>105.9513157894734</v>
       </c>
       <c r="Y24" s="12">
         <v>122.8</v>
       </c>
       <c r="Z24" s="23">
-        <v>-16.066118421052881</v>
+        <v>-16.84868421052656</v>
       </c>
       <c r="AA24" s="23">
-        <v>16.066118421052881</v>
+        <v>16.84868421052656</v>
       </c>
       <c r="AB24" s="24">
-        <v>13.08315832333296</v>
-      </c>
-    </row>
-    <row r="25" spans="2:28" x14ac:dyDescent="0.25">
+        <v>13.720426881536291</v>
+      </c>
+      <c r="AC24" s="32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B25" s="14" t="s">
         <v>4</v>
       </c>
@@ -1744,19 +1830,23 @@
         <v>5</v>
       </c>
       <c r="D25" s="25">
-        <v>11.52145000000003</v>
+        <v>11.793575000000031</v>
       </c>
       <c r="E25" s="25">
         <v>26.24</v>
       </c>
       <c r="F25" s="25">
-        <v>-14.71854999999996</v>
+        <v>-14.446424999999969</v>
       </c>
       <c r="G25" s="25">
-        <v>14.71854999999996</v>
+        <v>14.446424999999969</v>
       </c>
       <c r="H25" s="26">
-        <v>56.092035060975483</v>
+        <v>55.054973323170628</v>
+      </c>
+      <c r="I25" s="33">
+        <f>AVERAGE(H21:H25)</f>
+        <v>46.859643889293643</v>
       </c>
       <c r="L25" s="14" t="s">
         <v>4</v>
@@ -1765,19 +1855,23 @@
         <v>5</v>
       </c>
       <c r="N25" s="16">
-        <v>1.696505617283951</v>
+        <v>1.691573086419754</v>
       </c>
       <c r="O25" s="16">
         <v>1.5740000000000001</v>
       </c>
       <c r="P25" s="16">
-        <v>0.1225056172839509</v>
+        <v>0.11757308641975391</v>
       </c>
       <c r="Q25" s="16">
-        <v>0.1225056172839509</v>
+        <v>0.11757308641975391</v>
       </c>
       <c r="R25" s="26">
-        <v>7.7830760663247096</v>
+        <v>7.4697005349271883</v>
+      </c>
+      <c r="S25" s="33">
+        <f>AVERAGE(R21:R25)</f>
+        <v>6.9654320781238797</v>
       </c>
       <c r="V25" s="14" t="s">
         <v>4</v>
@@ -1786,22 +1880,26 @@
         <v>5</v>
       </c>
       <c r="X25" s="25">
-        <v>93.757072368421063</v>
+        <v>93.551151315789667</v>
       </c>
       <c r="Y25" s="15">
         <v>101.2</v>
       </c>
       <c r="Z25" s="25">
-        <v>-7.4429276315789394</v>
+        <v>-7.6488486842103356</v>
       </c>
       <c r="AA25" s="25">
-        <v>7.4429276315789394</v>
+        <v>7.6488486842103356</v>
       </c>
       <c r="AB25" s="26">
-        <v>7.3546715727064624</v>
-      </c>
-    </row>
-    <row r="26" spans="2:28" x14ac:dyDescent="0.25">
+        <v>7.5581508737256282</v>
+      </c>
+      <c r="AC25" s="33">
+        <f>AVERAGE(AB21:AB25)</f>
+        <v>7.5360483406472456</v>
+      </c>
+    </row>
+    <row r="26" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B26" s="2" t="s">
         <v>5</v>
       </c>
@@ -1809,19 +1907,19 @@
         <v>1</v>
       </c>
       <c r="D26" s="17">
-        <v>3.1136307716369629</v>
+        <v>3.931233167648315</v>
       </c>
       <c r="E26" s="17">
         <v>5.6</v>
       </c>
       <c r="F26" s="17">
-        <v>-2.4863692283630372</v>
+        <v>-1.668766832351684</v>
       </c>
       <c r="G26" s="17">
-        <v>2.4863692283630372</v>
+        <v>1.668766832351684</v>
       </c>
       <c r="H26" s="18">
-        <v>44.3994505064828</v>
+        <v>29.799407720565789</v>
       </c>
       <c r="L26" s="2" t="s">
         <v>5</v>
@@ -1830,19 +1928,19 @@
         <v>1</v>
       </c>
       <c r="N26" s="4">
-        <v>1.066467761993408</v>
+        <v>1.0792661905288701</v>
       </c>
       <c r="O26" s="4">
         <v>0.93700000000000006</v>
       </c>
       <c r="P26" s="4">
-        <v>0.12946776199340809</v>
+        <v>0.1422661905288696</v>
       </c>
       <c r="Q26" s="4">
-        <v>0.12946776199340809</v>
+        <v>0.1422661905288696</v>
       </c>
       <c r="R26" s="18">
-        <v>13.81726382000087</v>
+        <v>15.183158007350009</v>
       </c>
       <c r="V26" s="2" t="s">
         <v>5</v>
@@ -1851,22 +1949,22 @@
         <v>1</v>
       </c>
       <c r="X26" s="17">
-        <v>79.920700073242188</v>
+        <v>80.835586547851563</v>
       </c>
       <c r="Y26" s="3">
         <v>86.8</v>
       </c>
       <c r="Z26" s="17">
-        <v>-6.8792999267578097</v>
+        <v>-5.9644134521484347</v>
       </c>
       <c r="AA26" s="17">
-        <v>6.8792999267578097</v>
+        <v>5.9644134521484347</v>
       </c>
       <c r="AB26" s="18">
-        <v>7.9254607451126846</v>
-      </c>
-    </row>
-    <row r="27" spans="2:28" x14ac:dyDescent="0.25">
+        <v>6.8714440692954328</v>
+      </c>
+    </row>
+    <row r="27" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B27" s="5" t="s">
         <v>5</v>
       </c>
@@ -1874,19 +1972,19 @@
         <v>2</v>
       </c>
       <c r="D27" s="19">
-        <v>4.3806281089782706</v>
+        <v>4.0721087455749512</v>
       </c>
       <c r="E27" s="19">
         <v>5.47</v>
       </c>
       <c r="F27" s="19">
-        <v>-1.089371891021728</v>
+        <v>-1.397891254425049</v>
       </c>
       <c r="G27" s="19">
-        <v>1.089371891021728</v>
+        <v>1.397891254425049</v>
       </c>
       <c r="H27" s="20">
-        <v>19.915391060726289</v>
+        <v>25.555598801189191</v>
       </c>
       <c r="L27" s="5" t="s">
         <v>5</v>
@@ -1895,19 +1993,19 @@
         <v>2</v>
       </c>
       <c r="N27" s="7">
-        <v>0.90068113803863525</v>
+        <v>0.90371578931808472</v>
       </c>
       <c r="O27" s="7">
         <v>0.88400000000000001</v>
       </c>
       <c r="P27" s="7">
-        <v>1.6681138038635249E-2</v>
+        <v>1.9715789318084709E-2</v>
       </c>
       <c r="Q27" s="7">
-        <v>1.6681138038635249E-2</v>
+        <v>1.9715789318084709E-2</v>
       </c>
       <c r="R27" s="20">
-        <v>1.887006565456476</v>
+        <v>2.230292909285601</v>
       </c>
       <c r="V27" s="5" t="s">
         <v>5</v>
@@ -1916,22 +2014,22 @@
         <v>2</v>
       </c>
       <c r="X27" s="19">
-        <v>101.8134384155273</v>
+        <v>106.506706237793</v>
       </c>
       <c r="Y27" s="6">
         <v>106.9</v>
       </c>
       <c r="Z27" s="19">
-        <v>-5.0865615844726619</v>
+        <v>-0.39329376220703688</v>
       </c>
       <c r="AA27" s="19">
-        <v>5.0865615844726619</v>
+        <v>0.39329376220703688</v>
       </c>
       <c r="AB27" s="20">
-        <v>4.7582428292541268</v>
-      </c>
-    </row>
-    <row r="28" spans="2:28" x14ac:dyDescent="0.25">
+        <v>0.36790810309357991</v>
+      </c>
+    </row>
+    <row r="28" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B28" s="8" t="s">
         <v>5</v>
       </c>
@@ -1939,19 +2037,19 @@
         <v>3</v>
       </c>
       <c r="D28" s="21">
-        <v>17.59169769287109</v>
+        <v>16.629522323608398</v>
       </c>
       <c r="E28" s="21">
         <v>26.16</v>
       </c>
       <c r="F28" s="21">
-        <v>-8.5683023071289064</v>
+        <v>-9.5304776763916017</v>
       </c>
       <c r="G28" s="21">
-        <v>8.5683023071289064</v>
+        <v>9.5304776763916017</v>
       </c>
       <c r="H28" s="22">
-        <v>32.753449186272583</v>
+        <v>36.431489588652909</v>
       </c>
       <c r="L28" s="8" t="s">
         <v>5</v>
@@ -1960,19 +2058,19 @@
         <v>3</v>
       </c>
       <c r="N28" s="10">
-        <v>0.62977129220962524</v>
+        <v>0.54778569936752319</v>
       </c>
       <c r="O28" s="10">
         <v>0.60699999999999998</v>
       </c>
       <c r="P28" s="10">
-        <v>2.277129220962526E-2</v>
+        <v>-5.9214300632476791E-2</v>
       </c>
       <c r="Q28" s="10">
-        <v>2.277129220962526E-2</v>
+        <v>5.9214300632476791E-2</v>
       </c>
       <c r="R28" s="22">
-        <v>3.7514484694605041</v>
+        <v>9.7552389839335731</v>
       </c>
       <c r="V28" s="8" t="s">
         <v>5</v>
@@ -1981,22 +2079,22 @@
         <v>3</v>
       </c>
       <c r="X28" s="21">
-        <v>137.79722595214841</v>
+        <v>139.07914733886719</v>
       </c>
       <c r="Y28" s="9">
         <v>146.1</v>
       </c>
       <c r="Z28" s="21">
-        <v>-8.3027740478515568</v>
+        <v>-7.0208526611328068</v>
       </c>
       <c r="AA28" s="21">
-        <v>8.3027740478515568</v>
+        <v>7.0208526611328068</v>
       </c>
       <c r="AB28" s="22">
-        <v>5.6829391155725926</v>
-      </c>
-    </row>
-    <row r="29" spans="2:28" x14ac:dyDescent="0.25">
+        <v>4.8055117461552408</v>
+      </c>
+    </row>
+    <row r="29" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B29" s="11" t="s">
         <v>5</v>
       </c>
@@ -2004,19 +2102,22 @@
         <v>4</v>
       </c>
       <c r="D29" s="23">
-        <v>24.892646789550781</v>
+        <v>23.57191276550293</v>
       </c>
       <c r="E29" s="23">
         <v>47.29</v>
       </c>
       <c r="F29" s="23">
-        <v>-22.397353210449221</v>
+        <v>-23.718087234497069</v>
       </c>
       <c r="G29" s="23">
-        <v>22.397353210449221</v>
+        <v>23.718087234497069</v>
       </c>
       <c r="H29" s="24">
-        <v>47.361711166101117</v>
+        <v>50.15455114082696</v>
+      </c>
+      <c r="I29" s="32" t="s">
+        <v>17</v>
       </c>
       <c r="L29" s="11" t="s">
         <v>5</v>
@@ -2025,19 +2126,22 @@
         <v>4</v>
       </c>
       <c r="N29" s="13">
-        <v>0.81171232461929321</v>
+        <v>0.81157451868057251</v>
       </c>
       <c r="O29" s="13">
         <v>0.79400000000000004</v>
       </c>
       <c r="P29" s="13">
-        <v>1.771232461929317E-2</v>
+        <v>1.7574518680572471E-2</v>
       </c>
       <c r="Q29" s="13">
-        <v>1.771232461929317E-2</v>
+        <v>1.7574518680572471E-2</v>
       </c>
       <c r="R29" s="24">
-        <v>2.2307713626313821</v>
+        <v>2.2134154509537121</v>
+      </c>
+      <c r="S29" s="32" t="s">
+        <v>17</v>
       </c>
       <c r="V29" s="11" t="s">
         <v>5</v>
@@ -2046,22 +2150,25 @@
         <v>4</v>
       </c>
       <c r="X29" s="23">
-        <v>113.2471160888672</v>
+        <v>115.0807571411133</v>
       </c>
       <c r="Y29" s="12">
         <v>122.8</v>
       </c>
       <c r="Z29" s="23">
-        <v>-9.5528839111328097</v>
+        <v>-7.7192428588867159</v>
       </c>
       <c r="AA29" s="23">
-        <v>9.5528839111328097</v>
+        <v>7.7192428588867159</v>
       </c>
       <c r="AB29" s="24">
-        <v>7.7792214260039172</v>
-      </c>
-    </row>
-    <row r="30" spans="2:28" x14ac:dyDescent="0.25">
+        <v>6.2860283867155671</v>
+      </c>
+      <c r="AC29" s="32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B30" s="14" t="s">
         <v>5</v>
       </c>
@@ -2069,19 +2176,23 @@
         <v>5</v>
       </c>
       <c r="D30" s="25">
-        <v>11.53221225738525</v>
+        <v>11.19066715240479</v>
       </c>
       <c r="E30" s="25">
         <v>26.24</v>
       </c>
       <c r="F30" s="25">
-        <v>-14.707787742614739</v>
+        <v>-15.04933284759521</v>
       </c>
       <c r="G30" s="25">
-        <v>14.707787742614739</v>
+        <v>15.04933284759521</v>
       </c>
       <c r="H30" s="26">
-        <v>56.051020360574483</v>
+        <v>57.352640425286637</v>
+      </c>
+      <c r="I30" s="33">
+        <f>AVERAGE(H26:H30)</f>
+        <v>39.858737535304293</v>
       </c>
       <c r="L30" s="14" t="s">
         <v>5</v>
@@ -2090,19 +2201,23 @@
         <v>5</v>
       </c>
       <c r="N30" s="16">
-        <v>1.657795667648315</v>
+        <v>1.6652126312255859</v>
       </c>
       <c r="O30" s="16">
         <v>1.5740000000000001</v>
       </c>
       <c r="P30" s="16">
-        <v>8.3795667648315364E-2</v>
+        <v>9.1212631225585872E-2</v>
       </c>
       <c r="Q30" s="16">
-        <v>8.3795667648315364E-2</v>
+        <v>9.1212631225585872E-2</v>
       </c>
       <c r="R30" s="26">
-        <v>5.3237400030695916</v>
+        <v>5.7949575111553928</v>
+      </c>
+      <c r="S30" s="33">
+        <f>AVERAGE(R26:R30)</f>
+        <v>7.035412572535658</v>
       </c>
       <c r="V30" s="14" t="s">
         <v>5</v>
@@ -2111,42 +2226,46 @@
         <v>5</v>
       </c>
       <c r="X30" s="25">
-        <v>93.453887939453125</v>
+        <v>93.696861267089844</v>
       </c>
       <c r="Y30" s="15">
         <v>101.2</v>
       </c>
       <c r="Z30" s="25">
-        <v>-7.7461120605468778</v>
+        <v>-7.5031387329101591</v>
       </c>
       <c r="AA30" s="25">
-        <v>7.7461120605468778</v>
+        <v>7.5031387329101591</v>
       </c>
       <c r="AB30" s="26">
-        <v>7.6542609293941473</v>
-      </c>
-    </row>
-    <row r="34" spans="2:28" ht="18.75" x14ac:dyDescent="0.4">
+        <v>7.4141687084092469</v>
+      </c>
+      <c r="AC30" s="33">
+        <f>AVERAGE(AB26:AB30)</f>
+        <v>5.1490122027338128</v>
+      </c>
+    </row>
+    <row r="34" spans="2:29" ht="17.399999999999999" x14ac:dyDescent="0.45">
       <c r="D34" s="29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E34" s="30"/>
       <c r="F34" s="30"/>
       <c r="G34" s="31"/>
       <c r="N34" s="29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="O34" s="30"/>
       <c r="P34" s="30"/>
       <c r="Q34" s="31"/>
       <c r="X34" s="29" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="Y34" s="30"/>
       <c r="Z34" s="30"/>
       <c r="AA34" s="31"/>
     </row>
-    <row r="35" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B35" s="28" t="s">
         <v>0</v>
       </c>
@@ -2160,13 +2279,13 @@
         <v>3</v>
       </c>
       <c r="F35" s="28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G35" s="28" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="H35" s="28" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="L35" s="28" t="s">
         <v>0</v>
@@ -2181,13 +2300,13 @@
         <v>7</v>
       </c>
       <c r="P35" s="28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q35" s="28" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="R35" s="28" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="V35" s="28" t="s">
         <v>0</v>
@@ -2202,16 +2321,16 @@
         <v>9</v>
       </c>
       <c r="Z35" s="28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="AA35" s="28" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="AB35" s="28" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="36" spans="2:28" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="36" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B36" s="2" t="s">
         <v>4</v>
       </c>
@@ -2219,19 +2338,19 @@
         <v>1</v>
       </c>
       <c r="D36" s="17">
-        <v>3.95425</v>
+        <v>3.8371499999999998</v>
       </c>
       <c r="E36" s="17">
         <v>5.6</v>
       </c>
       <c r="F36" s="17">
-        <v>-1.64575</v>
+        <v>-1.76285</v>
       </c>
       <c r="G36" s="17">
-        <v>1.64575</v>
+        <v>1.76285</v>
       </c>
       <c r="H36" s="18">
-        <v>29.388392857142861</v>
+        <v>31.4794642857143</v>
       </c>
       <c r="L36" s="2" t="s">
         <v>4</v>
@@ -2240,19 +2359,19 @@
         <v>1</v>
       </c>
       <c r="N36" s="4">
-        <v>1.099679562289563</v>
+        <v>1.0832079761904769</v>
       </c>
       <c r="O36" s="4">
         <v>0.93700000000000006</v>
       </c>
       <c r="P36" s="4">
-        <v>0.1626795622895629</v>
+        <v>0.1462079761904769</v>
       </c>
       <c r="Q36" s="4">
-        <v>0.1626795622895629</v>
+        <v>0.1462079761904769</v>
       </c>
       <c r="R36" s="18">
-        <v>17.36174624221589</v>
+        <v>15.60383950805516</v>
       </c>
       <c r="V36" s="2" t="s">
         <v>4</v>
@@ -2261,22 +2380,22 @@
         <v>1</v>
       </c>
       <c r="X36" s="17">
-        <v>79.392598684210512</v>
+        <v>80.68009868421052</v>
       </c>
       <c r="Y36" s="3">
         <v>86.8</v>
       </c>
       <c r="Z36" s="17">
-        <v>-7.4074013157894854</v>
+        <v>-6.1199013157894768</v>
       </c>
       <c r="AA36" s="17">
-        <v>7.4074013157894854</v>
+        <v>6.1199013157894768</v>
       </c>
       <c r="AB36" s="18">
-        <v>8.5338724836284392</v>
-      </c>
-    </row>
-    <row r="37" spans="2:28" x14ac:dyDescent="0.25">
+        <v>7.0505775527528547</v>
+      </c>
+    </row>
+    <row r="37" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B37" s="5" t="s">
         <v>4</v>
       </c>
@@ -2284,19 +2403,19 @@
         <v>2</v>
       </c>
       <c r="D37" s="19">
-        <v>3.3723749999999968</v>
+        <v>3.3949250000000029</v>
       </c>
       <c r="E37" s="19">
         <v>5.47</v>
       </c>
       <c r="F37" s="19">
-        <v>-2.097625000000003</v>
+        <v>-2.0750749999999969</v>
       </c>
       <c r="G37" s="19">
-        <v>2.097625000000003</v>
+        <v>2.0750749999999969</v>
       </c>
       <c r="H37" s="20">
-        <v>38.347806215722173</v>
+        <v>37.935557586837227</v>
       </c>
       <c r="L37" s="5" t="s">
         <v>4</v>
@@ -2305,19 +2424,19 @@
         <v>2</v>
       </c>
       <c r="N37" s="7">
-        <v>0.89264339506172641</v>
+        <v>0.89449436948853378</v>
       </c>
       <c r="O37" s="7">
         <v>0.88400000000000001</v>
       </c>
       <c r="P37" s="7">
-        <v>8.6433950617263999E-3</v>
+        <v>1.0494369488533771E-2</v>
       </c>
       <c r="Q37" s="7">
-        <v>8.6433950617263999E-3</v>
+        <v>1.0494369488533771E-2</v>
       </c>
       <c r="R37" s="20">
-        <v>0.97775962236723979</v>
+        <v>1.187145869743639</v>
       </c>
       <c r="V37" s="5" t="s">
         <v>4</v>
@@ -2326,22 +2445,22 @@
         <v>2</v>
       </c>
       <c r="X37" s="19">
-        <v>104.3090460526315</v>
+        <v>104.5381578947368</v>
       </c>
       <c r="Y37" s="6">
         <v>106.9</v>
       </c>
       <c r="Z37" s="19">
-        <v>-2.5909539473685328</v>
+        <v>-2.3618421052632361</v>
       </c>
       <c r="AA37" s="19">
-        <v>2.5909539473685328</v>
+        <v>2.3618421052632361</v>
       </c>
       <c r="AB37" s="20">
-        <v>2.4237174437497968</v>
-      </c>
-    </row>
-    <row r="38" spans="2:28" x14ac:dyDescent="0.25">
+        <v>2.209393924474496</v>
+      </c>
+    </row>
+    <row r="38" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B38" s="8" t="s">
         <v>4</v>
       </c>
@@ -2349,19 +2468,19 @@
         <v>3</v>
       </c>
       <c r="D38" s="21">
-        <v>17.70522500000002</v>
+        <v>14.86860000000002</v>
       </c>
       <c r="E38" s="21">
         <v>26.16</v>
       </c>
       <c r="F38" s="21">
-        <v>-8.4547749999999837</v>
+        <v>-11.29139999999998</v>
       </c>
       <c r="G38" s="21">
-        <v>8.4547749999999837</v>
+        <v>11.29139999999998</v>
       </c>
       <c r="H38" s="22">
-        <v>32.319476299694131</v>
+        <v>43.162844036697159</v>
       </c>
       <c r="L38" s="8" t="s">
         <v>4</v>
@@ -2370,19 +2489,19 @@
         <v>3</v>
       </c>
       <c r="N38" s="10">
-        <v>0.63146691358024643</v>
+        <v>0.6568846913580243</v>
       </c>
       <c r="O38" s="10">
         <v>0.60699999999999998</v>
       </c>
       <c r="P38" s="10">
-        <v>2.4466913580246441E-2</v>
+        <v>4.9884691358024313E-2</v>
       </c>
       <c r="Q38" s="10">
-        <v>2.4466913580246441E-2</v>
+        <v>4.9884691358024313E-2</v>
       </c>
       <c r="R38" s="22">
-        <v>4.0307930115727251</v>
+        <v>8.2182358085707268</v>
       </c>
       <c r="V38" s="8" t="s">
         <v>4</v>
@@ -2391,22 +2510,22 @@
         <v>3</v>
       </c>
       <c r="X38" s="21">
-        <v>136.73865131578921</v>
+        <v>138.50624999999951</v>
       </c>
       <c r="Y38" s="9">
         <v>146.1</v>
       </c>
       <c r="Z38" s="21">
-        <v>-9.3613486842108102</v>
+        <v>-7.5937500000004547</v>
       </c>
       <c r="AA38" s="21">
-        <v>9.3613486842108102</v>
+        <v>7.5937500000004547</v>
       </c>
       <c r="AB38" s="22">
-        <v>6.4074939659211569</v>
-      </c>
-    </row>
-    <row r="39" spans="2:28" x14ac:dyDescent="0.25">
+        <v>5.1976386036964097</v>
+      </c>
+    </row>
+    <row r="39" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B39" s="11" t="s">
         <v>4</v>
       </c>
@@ -2414,19 +2533,22 @@
         <v>4</v>
       </c>
       <c r="D39" s="23">
-        <v>38.718525</v>
+        <v>36.657724999999957</v>
       </c>
       <c r="E39" s="23">
         <v>47.29</v>
       </c>
       <c r="F39" s="23">
-        <v>-8.5714749999999995</v>
+        <v>-10.632275000000041</v>
       </c>
       <c r="G39" s="23">
-        <v>8.5714749999999995</v>
+        <v>10.632275000000041</v>
       </c>
       <c r="H39" s="24">
-        <v>18.125343624444909</v>
+        <v>22.483135969549661</v>
+      </c>
+      <c r="I39" s="32" t="s">
+        <v>17</v>
       </c>
       <c r="L39" s="11" t="s">
         <v>4</v>
@@ -2435,19 +2557,22 @@
         <v>4</v>
       </c>
       <c r="N39" s="13">
-        <v>0.7505201234567892</v>
+        <v>0.7486531657848341</v>
       </c>
       <c r="O39" s="13">
         <v>0.79400000000000004</v>
       </c>
       <c r="P39" s="13">
-        <v>-4.3479876543210838E-2</v>
+        <v>-4.5346834215165943E-2</v>
       </c>
       <c r="Q39" s="13">
-        <v>4.3479876543210838E-2</v>
+        <v>4.5346834215165943E-2</v>
       </c>
       <c r="R39" s="24">
-        <v>5.4760549802532541</v>
+        <v>5.7111881883080526</v>
+      </c>
+      <c r="S39" s="32" t="s">
+        <v>17</v>
       </c>
       <c r="V39" s="11" t="s">
         <v>4</v>
@@ -2456,22 +2581,25 @@
         <v>4</v>
       </c>
       <c r="X39" s="23">
-        <v>99.646546052631464</v>
+        <v>99.757072368420978</v>
       </c>
       <c r="Y39" s="12">
         <v>122.8</v>
       </c>
       <c r="Z39" s="23">
-        <v>-23.153453947368529</v>
+        <v>-23.042927631579019</v>
       </c>
       <c r="AA39" s="23">
-        <v>23.153453947368529</v>
+        <v>23.042927631579019</v>
       </c>
       <c r="AB39" s="24">
-        <v>18.854604191668191</v>
-      </c>
-    </row>
-    <row r="40" spans="2:28" x14ac:dyDescent="0.25">
+        <v>18.76459904851712</v>
+      </c>
+      <c r="AC39" s="32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B40" s="14" t="s">
         <v>4</v>
       </c>
@@ -2479,19 +2607,23 @@
         <v>5</v>
       </c>
       <c r="D40" s="25">
-        <v>10.639225000000041</v>
+        <v>11.89877500000004</v>
       </c>
       <c r="E40" s="25">
         <v>26.24</v>
       </c>
       <c r="F40" s="25">
-        <v>-15.60077499999996</v>
+        <v>-14.341224999999961</v>
       </c>
       <c r="G40" s="25">
-        <v>15.60077499999996</v>
+        <v>14.341224999999961</v>
       </c>
       <c r="H40" s="26">
-        <v>59.454173018292543</v>
+        <v>54.654058689024247</v>
+      </c>
+      <c r="I40" s="33">
+        <f>AVERAGE(H36:H40)</f>
+        <v>37.943012113564521</v>
       </c>
       <c r="L40" s="14" t="s">
         <v>4</v>
@@ -2500,19 +2632,23 @@
         <v>5</v>
       </c>
       <c r="N40" s="16">
-        <v>1.676814673721339</v>
+        <v>1.6782232098765431</v>
       </c>
       <c r="O40" s="16">
         <v>1.5740000000000001</v>
       </c>
       <c r="P40" s="16">
-        <v>0.1028146737213389</v>
+        <v>0.1042232098765432</v>
       </c>
       <c r="Q40" s="16">
-        <v>0.1028146737213389</v>
+        <v>0.1042232098765432</v>
       </c>
       <c r="R40" s="26">
-        <v>6.5320631335031063</v>
+        <v>6.6215508180777123</v>
+      </c>
+      <c r="S40" s="33">
+        <f>AVERAGE(R36:R40)</f>
+        <v>7.4683920385510572</v>
       </c>
       <c r="V40" s="14" t="s">
         <v>4</v>
@@ -2521,22 +2657,26 @@
         <v>5</v>
       </c>
       <c r="X40" s="25">
-        <v>93.845723684210554</v>
+        <v>93.90476973684224</v>
       </c>
       <c r="Y40" s="15">
         <v>101.2</v>
       </c>
       <c r="Z40" s="25">
-        <v>-7.3542763157894484</v>
+        <v>-7.2952302631577624</v>
       </c>
       <c r="AA40" s="25">
-        <v>7.3542763157894484</v>
+        <v>7.2952302631577624</v>
       </c>
       <c r="AB40" s="26">
-        <v>7.2670714582899683</v>
-      </c>
-    </row>
-    <row r="41" spans="2:28" x14ac:dyDescent="0.25">
+        <v>7.2087255564800019</v>
+      </c>
+      <c r="AC40" s="33">
+        <f>AVERAGE(AB36:AB40)</f>
+        <v>8.086186937184177</v>
+      </c>
+    </row>
+    <row r="41" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B41" s="2" t="s">
         <v>5</v>
       </c>
@@ -2544,19 +2684,19 @@
         <v>1</v>
       </c>
       <c r="D41" s="17">
-        <v>4.4103779792785636</v>
+        <v>4.3981719017028809</v>
       </c>
       <c r="E41" s="17">
         <v>5.6</v>
       </c>
       <c r="F41" s="17">
-        <v>-1.189622020721435</v>
+        <v>-1.201828098297119</v>
       </c>
       <c r="G41" s="17">
-        <v>1.189622020721435</v>
+        <v>1.201828098297119</v>
       </c>
       <c r="H41" s="18">
-        <v>21.243250370025631</v>
+        <v>21.461216041019981</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>5</v>
@@ -2565,19 +2705,19 @@
         <v>1</v>
       </c>
       <c r="N41" s="4">
-        <v>1.1211763620376589</v>
+        <v>1.109668612480164</v>
       </c>
       <c r="O41" s="4">
         <v>0.93700000000000006</v>
       </c>
       <c r="P41" s="4">
-        <v>0.18417636203765861</v>
+        <v>0.17266861248016349</v>
       </c>
       <c r="Q41" s="4">
-        <v>0.18417636203765861</v>
+        <v>0.17266861248016349</v>
       </c>
       <c r="R41" s="18">
-        <v>19.655961796975301</v>
+        <v>18.42781349841659</v>
       </c>
       <c r="V41" s="2" t="s">
         <v>5</v>
@@ -2586,22 +2726,22 @@
         <v>1</v>
       </c>
       <c r="X41" s="17">
-        <v>74.600959777832031</v>
+        <v>78.849533081054688</v>
       </c>
       <c r="Y41" s="3">
         <v>86.8</v>
       </c>
       <c r="Z41" s="17">
-        <v>-12.199040222167969</v>
+        <v>-7.9504669189453097</v>
       </c>
       <c r="AA41" s="17">
-        <v>12.199040222167969</v>
+        <v>7.9504669189453097</v>
       </c>
       <c r="AB41" s="18">
-        <v>14.054193804340979</v>
-      </c>
-    </row>
-    <row r="42" spans="2:28" x14ac:dyDescent="0.25">
+        <v>9.1595241001674079</v>
+      </c>
+    </row>
+    <row r="42" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B42" s="5" t="s">
         <v>5</v>
       </c>
@@ -2609,19 +2749,19 @@
         <v>2</v>
       </c>
       <c r="D42" s="19">
-        <v>3.0259182453155522</v>
+        <v>3.1921343803405762</v>
       </c>
       <c r="E42" s="19">
         <v>5.47</v>
       </c>
       <c r="F42" s="19">
-        <v>-2.444081754684448</v>
+        <v>-2.277865619659424</v>
       </c>
       <c r="G42" s="19">
-        <v>2.444081754684448</v>
+        <v>2.277865619659424</v>
       </c>
       <c r="H42" s="20">
-        <v>44.681567727320797</v>
+        <v>41.642881529422738</v>
       </c>
       <c r="L42" s="5" t="s">
         <v>5</v>
@@ -2630,19 +2770,19 @@
         <v>2</v>
       </c>
       <c r="N42" s="7">
-        <v>0.93642622232437134</v>
+        <v>0.9327695369720459</v>
       </c>
       <c r="O42" s="7">
         <v>0.88400000000000001</v>
       </c>
       <c r="P42" s="7">
-        <v>5.242622232437133E-2</v>
+        <v>4.876953697204589E-2</v>
       </c>
       <c r="Q42" s="7">
-        <v>5.242622232437133E-2</v>
+        <v>4.876953697204589E-2</v>
       </c>
       <c r="R42" s="20">
-        <v>5.9305681362411011</v>
+        <v>5.5169159470640148</v>
       </c>
       <c r="V42" s="5" t="s">
         <v>5</v>
@@ -2651,22 +2791,22 @@
         <v>2</v>
       </c>
       <c r="X42" s="19">
-        <v>109.01576232910161</v>
+        <v>105.6653747558594</v>
       </c>
       <c r="Y42" s="6">
         <v>106.9</v>
       </c>
       <c r="Z42" s="19">
-        <v>2.1157623291015568</v>
+        <v>-1.2346252441406309</v>
       </c>
       <c r="AA42" s="19">
-        <v>2.1157623291015568</v>
+        <v>1.2346252441406309</v>
       </c>
       <c r="AB42" s="20">
-        <v>1.9791976885889211</v>
-      </c>
-    </row>
-    <row r="43" spans="2:28" x14ac:dyDescent="0.25">
+        <v>1.154934746623602</v>
+      </c>
+    </row>
+    <row r="43" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B43" s="8" t="s">
         <v>5</v>
       </c>
@@ -2674,19 +2814,19 @@
         <v>3</v>
       </c>
       <c r="D43" s="21">
-        <v>19.100053787231449</v>
+        <v>19.526510238647461</v>
       </c>
       <c r="E43" s="21">
         <v>26.16</v>
       </c>
       <c r="F43" s="21">
-        <v>-7.0599462127685548</v>
+        <v>-6.6334897613525392</v>
       </c>
       <c r="G43" s="21">
-        <v>7.0599462127685548</v>
+        <v>6.6334897613525392</v>
       </c>
       <c r="H43" s="22">
-        <v>26.987561975414959</v>
+        <v>25.357376763580039</v>
       </c>
       <c r="L43" s="8" t="s">
         <v>5</v>
@@ -2695,19 +2835,19 @@
         <v>3</v>
       </c>
       <c r="N43" s="10">
-        <v>0.64759188890457153</v>
+        <v>0.61175382137298584</v>
       </c>
       <c r="O43" s="10">
         <v>0.60699999999999998</v>
       </c>
       <c r="P43" s="10">
-        <v>4.0591888904571549E-2</v>
+        <v>4.7538213729858558E-3</v>
       </c>
       <c r="Q43" s="10">
-        <v>4.0591888904571549E-2</v>
+        <v>4.7538213729858558E-3</v>
       </c>
       <c r="R43" s="22">
-        <v>6.6872963598964663</v>
+        <v>0.78316661828432554</v>
       </c>
       <c r="V43" s="8" t="s">
         <v>5</v>
@@ -2716,22 +2856,22 @@
         <v>3</v>
       </c>
       <c r="X43" s="21">
-        <v>144.29133605957031</v>
+        <v>142.3410339355469</v>
       </c>
       <c r="Y43" s="9">
         <v>146.1</v>
       </c>
       <c r="Z43" s="21">
-        <v>-1.808663940429682</v>
+        <v>-3.7589660644531189</v>
       </c>
       <c r="AA43" s="21">
-        <v>1.808663940429682</v>
+        <v>3.7589660644531189</v>
       </c>
       <c r="AB43" s="22">
-        <v>1.237962998240713</v>
-      </c>
-    </row>
-    <row r="44" spans="2:28" x14ac:dyDescent="0.25">
+        <v>2.572872049591457</v>
+      </c>
+    </row>
+    <row r="44" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B44" s="11" t="s">
         <v>5</v>
       </c>
@@ -2739,19 +2879,22 @@
         <v>4</v>
       </c>
       <c r="D44" s="23">
-        <v>33.822059631347663</v>
+        <v>39.949951171875</v>
       </c>
       <c r="E44" s="23">
         <v>47.29</v>
       </c>
       <c r="F44" s="23">
-        <v>-13.467940368652339</v>
+        <v>-7.3400488281249991</v>
       </c>
       <c r="G44" s="23">
-        <v>13.467940368652339</v>
+        <v>7.3400488281249991</v>
       </c>
       <c r="H44" s="24">
-        <v>28.479467897340541</v>
+        <v>15.52135510282301</v>
+      </c>
+      <c r="I44" s="32" t="s">
+        <v>17</v>
       </c>
       <c r="L44" s="11" t="s">
         <v>5</v>
@@ -2760,19 +2903,22 @@
         <v>4</v>
       </c>
       <c r="N44" s="13">
-        <v>0.69600147008895874</v>
+        <v>0.73988860845565796</v>
       </c>
       <c r="O44" s="13">
         <v>0.79400000000000004</v>
       </c>
       <c r="P44" s="13">
-        <v>-9.7998529911041299E-2</v>
+        <v>-5.411139154434208E-2</v>
       </c>
       <c r="Q44" s="13">
-        <v>9.7998529911041299E-2</v>
+        <v>5.411139154434208E-2</v>
       </c>
       <c r="R44" s="24">
-        <v>12.342384119778499</v>
+        <v>6.8150367184309921</v>
+      </c>
+      <c r="S44" s="32" t="s">
+        <v>17</v>
       </c>
       <c r="V44" s="11" t="s">
         <v>5</v>
@@ -2781,22 +2927,25 @@
         <v>4</v>
       </c>
       <c r="X44" s="23">
-        <v>107.0491409301758</v>
+        <v>111.6286544799805</v>
       </c>
       <c r="Y44" s="12">
         <v>122.8</v>
       </c>
       <c r="Z44" s="23">
-        <v>-15.750859069824219</v>
+        <v>-11.17134552001953</v>
       </c>
       <c r="AA44" s="23">
-        <v>15.750859069824219</v>
+        <v>11.17134552001953</v>
       </c>
       <c r="AB44" s="24">
-        <v>12.82643246728356</v>
-      </c>
-    </row>
-    <row r="45" spans="2:28" x14ac:dyDescent="0.25">
+        <v>9.0971869055533627</v>
+      </c>
+      <c r="AC44" s="32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="45" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B45" s="14" t="s">
         <v>5</v>
       </c>
@@ -2804,19 +2953,23 @@
         <v>5</v>
       </c>
       <c r="D45" s="25">
-        <v>10.161393165588381</v>
+        <v>10.19211483001709</v>
       </c>
       <c r="E45" s="25">
         <v>26.24</v>
       </c>
       <c r="F45" s="25">
-        <v>-16.07860683441162</v>
+        <v>-16.047885169982909</v>
       </c>
       <c r="G45" s="25">
-        <v>16.07860683441162</v>
+        <v>16.047885169982909</v>
       </c>
       <c r="H45" s="26">
-        <v>61.275178484800378</v>
+        <v>61.158098970971452</v>
+      </c>
+      <c r="I45" s="33">
+        <f>AVERAGE(H41:H45)</f>
+        <v>33.028185681563443</v>
       </c>
       <c r="L45" s="14" t="s">
         <v>5</v>
@@ -2825,19 +2978,23 @@
         <v>5</v>
       </c>
       <c r="N45" s="16">
-        <v>1.664501428604126</v>
+        <v>1.6732498407363889</v>
       </c>
       <c r="O45" s="16">
         <v>1.5740000000000001</v>
       </c>
       <c r="P45" s="16">
-        <v>9.0501428604125911E-2</v>
+        <v>9.9249840736389094E-2</v>
       </c>
       <c r="Q45" s="16">
-        <v>9.0501428604125911E-2</v>
+        <v>9.9249840736389094E-2</v>
       </c>
       <c r="R45" s="26">
-        <v>5.7497731006433241</v>
+        <v>6.3055807329345042</v>
+      </c>
+      <c r="S45" s="33">
+        <f>AVERAGE(R41:R45)</f>
+        <v>7.5697027030260857</v>
       </c>
       <c r="V45" s="14" t="s">
         <v>5</v>
@@ -2846,19 +3003,23 @@
         <v>5</v>
       </c>
       <c r="X45" s="25">
-        <v>93.185890197753906</v>
+        <v>93.882156372070313</v>
       </c>
       <c r="Y45" s="15">
         <v>101.2</v>
       </c>
       <c r="Z45" s="25">
-        <v>-8.0141098022460966</v>
+        <v>-7.3178436279296903</v>
       </c>
       <c r="AA45" s="25">
-        <v>8.0141098022460966</v>
+        <v>7.3178436279296903</v>
       </c>
       <c r="AB45" s="26">
-        <v>7.9190808322589881</v>
+        <v>7.2310707785866501</v>
+      </c>
+      <c r="AC45" s="33">
+        <f>AVERAGE(AB41:AB45)</f>
+        <v>5.843117716104496</v>
       </c>
     </row>
   </sheetData>

</xml_diff>